<commit_message>
feat: cadastrar 29 produtos no catálogo e estoque de peças
- 28 novos produtos + Polvo atualizado
- Estoque com quantidades informadas (360 peças total)
- Categorias, filamentos, horas e precificação automática
- Named range Produtos atualizado para dropdown do Romaneio

Co-authored-by: juanfazolo-cpu <juanfazolo-cpu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/taldo_gestao_v7.3.xlsx
+++ b/taldo_gestao_v7.3.xlsx
@@ -19,7 +19,7 @@
     <sheet name="📊 Resumo Parcelas" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="Produtos">'📋 Catálogo'!$B$7:$B$11</definedName>
+    <definedName name="Produtos">'📋 Catálogo'!$B$7:$B$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -17636,7 +17636,7 @@
       </c>
       <c r="B11" s="32" t="inlineStr">
         <is>
-          <t>Miniatura Polvo</t>
+          <t>Polvo</t>
         </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
@@ -17706,7 +17706,11 @@
         <v/>
       </c>
       <c r="T11" s="91" t="n"/>
-      <c r="U11" s="43" t="n"/>
+      <c r="U11" s="43" t="inlineStr">
+        <is>
+          <t>Estoque: 12 un</t>
+        </is>
+      </c>
       <c r="V11" s="0">
         <f>IF(B11="","",IFERROR(VLOOKUP(C11,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B11,B11),"000"),""))</f>
         <v/>
@@ -17717,19 +17721,57 @@
         <f>IF(T12="","",IMAGE(T12,4,50,50))</f>
         <v/>
       </c>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="47" t="n"/>
-      <c r="F12" s="48" t="n"/>
-      <c r="G12" s="47" t="n"/>
-      <c r="H12" s="48" t="n"/>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Estádio Corinthians</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Preto e Branco</t>
+        </is>
+      </c>
+      <c r="E12" s="47" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="F12" s="48" t="n">
+        <v>35</v>
+      </c>
+      <c r="G12" s="47" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="H12" s="48" t="n">
+        <v>20</v>
+      </c>
       <c r="I12" s="47" t="n"/>
       <c r="J12" s="48" t="n"/>
-      <c r="K12" s="49" t="n"/>
-      <c r="L12" s="46" t="n"/>
-      <c r="M12" s="46" t="n"/>
-      <c r="N12" s="46" t="n"/>
+      <c r="K12" s="49" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L12" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M12" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N12" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O12" s="50" t="n"/>
       <c r="P12" s="51" t="n"/>
       <c r="Q12" s="39">
@@ -17745,7 +17787,11 @@
         <v/>
       </c>
       <c r="T12" s="91" t="n"/>
-      <c r="U12" s="52" t="n"/>
+      <c r="U12" s="52" t="inlineStr">
+        <is>
+          <t>Estádio time Corinthians</t>
+        </is>
+      </c>
       <c r="V12" s="0">
         <f>IF(B12="","",IFERROR(VLOOKUP(C12,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B12,B12),"000"),""))</f>
         <v/>
@@ -17756,19 +17802,57 @@
         <f>IF(T13="","",IMAGE(T13,4,50,50))</f>
         <v/>
       </c>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="34" t="n"/>
-      <c r="F13" s="35" t="n"/>
-      <c r="G13" s="34" t="n"/>
-      <c r="H13" s="35" t="n"/>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Estádio Palmeiras</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Verde e Branco</t>
+        </is>
+      </c>
+      <c r="E13" s="34" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="F13" s="35" t="n">
+        <v>40</v>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="H13" s="35" t="n">
+        <v>15</v>
+      </c>
       <c r="I13" s="34" t="n"/>
       <c r="J13" s="35" t="n"/>
-      <c r="K13" s="36" t="n"/>
-      <c r="L13" s="33" t="n"/>
-      <c r="M13" s="33" t="n"/>
-      <c r="N13" s="33" t="n"/>
+      <c r="K13" s="36" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L13" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M13" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N13" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O13" s="37" t="n"/>
       <c r="P13" s="38" t="n"/>
       <c r="Q13" s="39">
@@ -17784,7 +17868,11 @@
         <v/>
       </c>
       <c r="T13" s="91" t="n"/>
-      <c r="U13" s="43" t="n"/>
+      <c r="U13" s="43" t="inlineStr">
+        <is>
+          <t>Estádio time Palmeiras</t>
+        </is>
+      </c>
       <c r="V13" s="0">
         <f>IF(B13="","",IFERROR(VLOOKUP(C13,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B13,B13),"000"),""))</f>
         <v/>
@@ -17795,19 +17883,63 @@
         <f>IF(T14="","",IMAGE(T14,4,50,50))</f>
         <v/>
       </c>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="47" t="n"/>
-      <c r="F14" s="48" t="n"/>
-      <c r="G14" s="47" t="n"/>
-      <c r="H14" s="48" t="n"/>
-      <c r="I14" s="47" t="n"/>
-      <c r="J14" s="48" t="n"/>
-      <c r="K14" s="49" t="n"/>
-      <c r="L14" s="46" t="n"/>
-      <c r="M14" s="46" t="n"/>
-      <c r="N14" s="46" t="n"/>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Estádio São Paulo</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Vermelho, Branco e Preto</t>
+        </is>
+      </c>
+      <c r="E14" s="47" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="F14" s="48" t="n">
+        <v>25</v>
+      </c>
+      <c r="G14" s="47" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="H14" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="I14" s="47" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="J14" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" s="49" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L14" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M14" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N14" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O14" s="50" t="n"/>
       <c r="P14" s="51" t="n"/>
       <c r="Q14" s="39">
@@ -17823,7 +17955,11 @@
         <v/>
       </c>
       <c r="T14" s="91" t="n"/>
-      <c r="U14" s="52" t="n"/>
+      <c r="U14" s="52" t="inlineStr">
+        <is>
+          <t>Estádio time São Paulo</t>
+        </is>
+      </c>
       <c r="V14" s="0">
         <f>IF(B14="","",IFERROR(VLOOKUP(C14,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B14,B14),"000"),""))</f>
         <v/>
@@ -17834,19 +17970,51 @@
         <f>IF(T15="","",IMAGE(T15,4,50,50))</f>
         <v/>
       </c>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="34" t="n"/>
-      <c r="F15" s="35" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Martelo Thor</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Cinza e Prata</t>
+        </is>
+      </c>
+      <c r="E15" s="34" t="inlineStr">
+        <is>
+          <t>Cinza</t>
+        </is>
+      </c>
+      <c r="F15" s="35" t="n">
+        <v>30</v>
+      </c>
       <c r="G15" s="34" t="n"/>
       <c r="H15" s="35" t="n"/>
       <c r="I15" s="34" t="n"/>
       <c r="J15" s="35" t="n"/>
-      <c r="K15" s="36" t="n"/>
-      <c r="L15" s="33" t="n"/>
-      <c r="M15" s="33" t="n"/>
-      <c r="N15" s="33" t="n"/>
+      <c r="K15" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="L15" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M15" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N15" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O15" s="37" t="n"/>
       <c r="P15" s="38" t="n"/>
       <c r="Q15" s="39">
@@ -17862,7 +18030,11 @@
         <v/>
       </c>
       <c r="T15" s="91" t="n"/>
-      <c r="U15" s="43" t="n"/>
+      <c r="U15" s="43" t="inlineStr">
+        <is>
+          <t>Martelo do Thor</t>
+        </is>
+      </c>
       <c r="V15" s="0">
         <f>IF(B15="","",IFERROR(VLOOKUP(C15,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B15,B15),"000"),""))</f>
         <v/>
@@ -17873,19 +18045,57 @@
         <f>IF(T16="","",IMAGE(T16,4,50,50))</f>
         <v/>
       </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="47" t="n"/>
-      <c r="F16" s="48" t="n"/>
-      <c r="G16" s="47" t="n"/>
-      <c r="H16" s="48" t="n"/>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Estádio Santos</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Branco e Preto</t>
+        </is>
+      </c>
+      <c r="E16" s="47" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="F16" s="48" t="n">
+        <v>35</v>
+      </c>
+      <c r="G16" s="47" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="H16" s="48" t="n">
+        <v>15</v>
+      </c>
       <c r="I16" s="47" t="n"/>
       <c r="J16" s="48" t="n"/>
-      <c r="K16" s="49" t="n"/>
-      <c r="L16" s="46" t="n"/>
-      <c r="M16" s="46" t="n"/>
-      <c r="N16" s="46" t="n"/>
+      <c r="K16" s="49" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L16" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M16" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N16" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O16" s="50" t="n"/>
       <c r="P16" s="51" t="n"/>
       <c r="Q16" s="39">
@@ -17901,7 +18111,11 @@
         <v/>
       </c>
       <c r="T16" s="91" t="n"/>
-      <c r="U16" s="52" t="n"/>
+      <c r="U16" s="52" t="inlineStr">
+        <is>
+          <t>Estádio time Santos</t>
+        </is>
+      </c>
       <c r="V16" s="0">
         <f>IF(B16="","",IFERROR(VLOOKUP(C16,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B16,B16),"000"),""))</f>
         <v/>
@@ -17912,19 +18126,57 @@
         <f>IF(T17="","",IMAGE(T17,4,50,50))</f>
         <v/>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="34" t="n"/>
-      <c r="F17" s="35" t="n"/>
-      <c r="G17" s="34" t="n"/>
-      <c r="H17" s="35" t="n"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Estádio Flamengo</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Vermelho e Preto</t>
+        </is>
+      </c>
+      <c r="E17" s="34" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="F17" s="35" t="n">
+        <v>35</v>
+      </c>
+      <c r="G17" s="34" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="H17" s="35" t="n">
+        <v>15</v>
+      </c>
       <c r="I17" s="34" t="n"/>
       <c r="J17" s="35" t="n"/>
-      <c r="K17" s="36" t="n"/>
-      <c r="L17" s="33" t="n"/>
-      <c r="M17" s="33" t="n"/>
-      <c r="N17" s="33" t="n"/>
+      <c r="K17" s="36" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L17" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M17" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N17" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O17" s="37" t="n"/>
       <c r="P17" s="38" t="n"/>
       <c r="Q17" s="39">
@@ -17940,7 +18192,11 @@
         <v/>
       </c>
       <c r="T17" s="91" t="n"/>
-      <c r="U17" s="43" t="n"/>
+      <c r="U17" s="43" t="inlineStr">
+        <is>
+          <t>Estádio time Flamengo</t>
+        </is>
+      </c>
       <c r="V17" s="0">
         <f>IF(B17="","",IFERROR(VLOOKUP(C17,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B17,B17),"000"),""))</f>
         <v/>
@@ -17951,19 +18207,57 @@
         <f>IF(T18="","",IMAGE(T18,4,50,50))</f>
         <v/>
       </c>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="47" t="n"/>
-      <c r="F18" s="48" t="n"/>
-      <c r="G18" s="47" t="n"/>
-      <c r="H18" s="48" t="n"/>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Escudo Flamengo</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Vermelho e Preto</t>
+        </is>
+      </c>
+      <c r="E18" s="47" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="F18" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="47" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="H18" s="48" t="n">
+        <v>5</v>
+      </c>
       <c r="I18" s="47" t="n"/>
       <c r="J18" s="48" t="n"/>
-      <c r="K18" s="49" t="n"/>
-      <c r="L18" s="46" t="n"/>
-      <c r="M18" s="46" t="n"/>
-      <c r="N18" s="46" t="n"/>
+      <c r="K18" s="49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L18" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M18" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N18" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O18" s="50" t="n"/>
       <c r="P18" s="51" t="n"/>
       <c r="Q18" s="39">
@@ -17979,7 +18273,11 @@
         <v/>
       </c>
       <c r="T18" s="91" t="n"/>
-      <c r="U18" s="52" t="n"/>
+      <c r="U18" s="52" t="inlineStr">
+        <is>
+          <t>Escudo time Flamengo</t>
+        </is>
+      </c>
       <c r="V18" s="0">
         <f>IF(B18="","",IFERROR(VLOOKUP(C18,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B18,B18),"000"),""))</f>
         <v/>
@@ -17990,19 +18288,63 @@
         <f>IF(T19="","",IMAGE(T19,4,50,50))</f>
         <v/>
       </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="34" t="n"/>
-      <c r="F19" s="35" t="n"/>
-      <c r="G19" s="34" t="n"/>
-      <c r="H19" s="35" t="n"/>
-      <c r="I19" s="34" t="n"/>
-      <c r="J19" s="35" t="n"/>
-      <c r="K19" s="36" t="n"/>
-      <c r="L19" s="33" t="n"/>
-      <c r="M19" s="33" t="n"/>
-      <c r="N19" s="33" t="n"/>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Estela Sensorial Maior</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Multicolor</t>
+        </is>
+      </c>
+      <c r="E19" s="34" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="F19" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G19" s="34" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="H19" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I19" s="34" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="J19" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="K19" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="L19" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M19" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N19" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O19" s="37" t="n"/>
       <c r="P19" s="38" t="n"/>
       <c r="Q19" s="39">
@@ -18018,7 +18360,11 @@
         <v/>
       </c>
       <c r="T19" s="91" t="n"/>
-      <c r="U19" s="43" t="n"/>
+      <c r="U19" s="43" t="inlineStr">
+        <is>
+          <t>Peça sensorial — modelo maior</t>
+        </is>
+      </c>
       <c r="V19" s="0">
         <f>IF(B19="","",IFERROR(VLOOKUP(C19,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B19,B19),"000"),""))</f>
         <v/>
@@ -18029,19 +18375,51 @@
         <f>IF(T20="","",IMAGE(T20,4,50,50))</f>
         <v/>
       </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="47" t="n"/>
-      <c r="F20" s="48" t="n"/>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Minicraft Verde</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="E20" s="47" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="F20" s="48" t="n">
+        <v>18</v>
+      </c>
       <c r="G20" s="47" t="n"/>
       <c r="H20" s="48" t="n"/>
       <c r="I20" s="47" t="n"/>
       <c r="J20" s="48" t="n"/>
-      <c r="K20" s="49" t="n"/>
-      <c r="L20" s="46" t="n"/>
-      <c r="M20" s="46" t="n"/>
-      <c r="N20" s="46" t="n"/>
+      <c r="K20" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M20" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N20" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O20" s="50" t="n"/>
       <c r="P20" s="51" t="n"/>
       <c r="Q20" s="39">
@@ -18057,7 +18435,11 @@
         <v/>
       </c>
       <c r="T20" s="91" t="n"/>
-      <c r="U20" s="52" t="n"/>
+      <c r="U20" s="52" t="inlineStr">
+        <is>
+          <t>Estilo Minecraft</t>
+        </is>
+      </c>
       <c r="V20" s="0">
         <f>IF(B20="","",IFERROR(VLOOKUP(C20,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B20,B20),"000"),""))</f>
         <v/>
@@ -18068,19 +18450,63 @@
         <f>IF(T21="","",IMAGE(T21,4,50,50))</f>
         <v/>
       </c>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="34" t="n"/>
-      <c r="F21" s="35" t="n"/>
-      <c r="G21" s="34" t="n"/>
-      <c r="H21" s="35" t="n"/>
-      <c r="I21" s="34" t="n"/>
-      <c r="J21" s="35" t="n"/>
-      <c r="K21" s="36" t="n"/>
-      <c r="L21" s="33" t="n"/>
-      <c r="M21" s="33" t="n"/>
-      <c r="N21" s="33" t="n"/>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Pentágono Sensorial</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Multicolor</t>
+        </is>
+      </c>
+      <c r="E21" s="34" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="F21" s="35" t="n">
+        <v>12</v>
+      </c>
+      <c r="G21" s="34" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="H21" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="I21" s="34" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="J21" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="K21" s="36" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L21" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M21" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N21" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O21" s="37" t="n"/>
       <c r="P21" s="38" t="n"/>
       <c r="Q21" s="39">
@@ -18096,7 +18522,11 @@
         <v/>
       </c>
       <c r="T21" s="91" t="n"/>
-      <c r="U21" s="43" t="n"/>
+      <c r="U21" s="43" t="inlineStr">
+        <is>
+          <t>Peça sensorial pentágono</t>
+        </is>
+      </c>
       <c r="V21" s="0">
         <f>IF(B21="","",IFERROR(VLOOKUP(C21,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B21,B21),"000"),""))</f>
         <v/>
@@ -18107,19 +18537,57 @@
         <f>IF(T22="","",IMAGE(T22,4,50,50))</f>
         <v/>
       </c>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="47" t="n"/>
-      <c r="F22" s="48" t="n"/>
-      <c r="G22" s="47" t="n"/>
-      <c r="H22" s="48" t="n"/>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Tubarão</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Cinza e Azul</t>
+        </is>
+      </c>
+      <c r="E22" s="47" t="inlineStr">
+        <is>
+          <t>Cinza</t>
+        </is>
+      </c>
+      <c r="F22" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="G22" s="47" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="H22" s="48" t="n">
+        <v>8</v>
+      </c>
       <c r="I22" s="47" t="n"/>
       <c r="J22" s="48" t="n"/>
-      <c r="K22" s="49" t="n"/>
-      <c r="L22" s="46" t="n"/>
-      <c r="M22" s="46" t="n"/>
-      <c r="N22" s="46" t="n"/>
+      <c r="K22" s="49" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L22" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M22" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N22" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O22" s="50" t="n"/>
       <c r="P22" s="51" t="n"/>
       <c r="Q22" s="39">
@@ -18146,19 +18614,57 @@
         <f>IF(T23="","",IMAGE(T23,4,50,50))</f>
         <v/>
       </c>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="34" t="n"/>
-      <c r="F23" s="35" t="n"/>
-      <c r="G23" s="34" t="n"/>
-      <c r="H23" s="35" t="n"/>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Nossa Senhora</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Branco e Azul</t>
+        </is>
+      </c>
+      <c r="E23" s="34" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="F23" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="G23" s="34" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="H23" s="35" t="n">
+        <v>5</v>
+      </c>
       <c r="I23" s="34" t="n"/>
       <c r="J23" s="35" t="n"/>
-      <c r="K23" s="36" t="n"/>
-      <c r="L23" s="33" t="n"/>
-      <c r="M23" s="33" t="n"/>
-      <c r="N23" s="33" t="n"/>
+      <c r="K23" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="L23" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M23" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N23" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O23" s="37" t="n"/>
       <c r="P23" s="38" t="n"/>
       <c r="Q23" s="39">
@@ -18174,7 +18680,11 @@
         <v/>
       </c>
       <c r="T23" s="91" t="n"/>
-      <c r="U23" s="43" t="n"/>
+      <c r="U23" s="43" t="inlineStr">
+        <is>
+          <t>Imagem religiosa</t>
+        </is>
+      </c>
       <c r="V23" s="0">
         <f>IF(B23="","",IFERROR(VLOOKUP(C23,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B23,B23),"000"),""))</f>
         <v/>
@@ -18185,19 +18695,51 @@
         <f>IF(T24="","",IMAGE(T24,4,50,50))</f>
         <v/>
       </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="47" t="n"/>
-      <c r="F24" s="48" t="n"/>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Gato Preto</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="E24" s="47" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="F24" s="48" t="n">
+        <v>15</v>
+      </c>
       <c r="G24" s="47" t="n"/>
       <c r="H24" s="48" t="n"/>
       <c r="I24" s="47" t="n"/>
       <c r="J24" s="48" t="n"/>
-      <c r="K24" s="49" t="n"/>
-      <c r="L24" s="46" t="n"/>
-      <c r="M24" s="46" t="n"/>
-      <c r="N24" s="46" t="n"/>
+      <c r="K24" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M24" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N24" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O24" s="50" t="n"/>
       <c r="P24" s="51" t="n"/>
       <c r="Q24" s="39">
@@ -18224,19 +18766,51 @@
         <f>IF(T25="","",IMAGE(T25,4,50,50))</f>
         <v/>
       </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="34" t="n"/>
-      <c r="F25" s="35" t="n"/>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Stormtrooper</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="E25" s="34" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="F25" s="35" t="n">
+        <v>22</v>
+      </c>
       <c r="G25" s="34" t="n"/>
       <c r="H25" s="35" t="n"/>
       <c r="I25" s="34" t="n"/>
       <c r="J25" s="35" t="n"/>
-      <c r="K25" s="36" t="n"/>
-      <c r="L25" s="33" t="n"/>
-      <c r="M25" s="33" t="n"/>
-      <c r="N25" s="33" t="n"/>
+      <c r="K25" s="36" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L25" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M25" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N25" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O25" s="37" t="n"/>
       <c r="P25" s="38" t="n"/>
       <c r="Q25" s="39">
@@ -18252,7 +18826,11 @@
         <v/>
       </c>
       <c r="T25" s="91" t="n"/>
-      <c r="U25" s="43" t="n"/>
+      <c r="U25" s="43" t="inlineStr">
+        <is>
+          <t>Star Wars</t>
+        </is>
+      </c>
       <c r="V25" s="0">
         <f>IF(B25="","",IFERROR(VLOOKUP(C25,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B25,B25),"000"),""))</f>
         <v/>
@@ -18263,19 +18841,51 @@
         <f>IF(T26="","",IMAGE(T26,4,50,50))</f>
         <v/>
       </c>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="47" t="n"/>
-      <c r="F26" s="48" t="n"/>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Copo Stanley</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="E26" s="47" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="F26" s="48" t="n">
+        <v>12</v>
+      </c>
       <c r="G26" s="47" t="n"/>
       <c r="H26" s="48" t="n"/>
       <c r="I26" s="47" t="n"/>
       <c r="J26" s="48" t="n"/>
-      <c r="K26" s="49" t="n"/>
-      <c r="L26" s="46" t="n"/>
-      <c r="M26" s="46" t="n"/>
-      <c r="N26" s="46" t="n"/>
+      <c r="K26" s="49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L26" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M26" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N26" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O26" s="50" t="n"/>
       <c r="P26" s="51" t="n"/>
       <c r="Q26" s="39">
@@ -18291,7 +18901,11 @@
         <v/>
       </c>
       <c r="T26" s="91" t="n"/>
-      <c r="U26" s="52" t="n"/>
+      <c r="U26" s="52" t="inlineStr">
+        <is>
+          <t>Base/suporte copo Stanley</t>
+        </is>
+      </c>
       <c r="V26" s="0">
         <f>IF(B26="","",IFERROR(VLOOKUP(C26,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B26,B26),"000"),""))</f>
         <v/>
@@ -18302,19 +18916,57 @@
         <f>IF(T27="","",IMAGE(T27,4,50,50))</f>
         <v/>
       </c>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
-      <c r="E27" s="34" t="n"/>
-      <c r="F27" s="35" t="n"/>
-      <c r="G27" s="34" t="n"/>
-      <c r="H27" s="35" t="n"/>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Homem de Ferro</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Vermelho e Dourado</t>
+        </is>
+      </c>
+      <c r="E27" s="34" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="F27" s="35" t="n">
+        <v>18</v>
+      </c>
+      <c r="G27" s="34" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="H27" s="35" t="n">
+        <v>7</v>
+      </c>
       <c r="I27" s="34" t="n"/>
       <c r="J27" s="35" t="n"/>
-      <c r="K27" s="36" t="n"/>
-      <c r="L27" s="33" t="n"/>
-      <c r="M27" s="33" t="n"/>
-      <c r="N27" s="33" t="n"/>
+      <c r="K27" s="36" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L27" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M27" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N27" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O27" s="37" t="n"/>
       <c r="P27" s="38" t="n"/>
       <c r="Q27" s="39">
@@ -18330,7 +18982,11 @@
         <v/>
       </c>
       <c r="T27" s="91" t="n"/>
-      <c r="U27" s="43" t="n"/>
+      <c r="U27" s="43" t="inlineStr">
+        <is>
+          <t>Marvel</t>
+        </is>
+      </c>
       <c r="V27" s="0">
         <f>IF(B27="","",IFERROR(VLOOKUP(C27,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B27,B27),"000"),""))</f>
         <v/>
@@ -18341,19 +18997,57 @@
         <f>IF(T28="","",IMAGE(T28,4,50,50))</f>
         <v/>
       </c>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="47" t="n"/>
-      <c r="F28" s="48" t="n"/>
-      <c r="G28" s="47" t="n"/>
-      <c r="H28" s="48" t="n"/>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Homem Aranha</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Vermelho e Azul</t>
+        </is>
+      </c>
+      <c r="E28" s="47" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="F28" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="G28" s="47" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="H28" s="48" t="n">
+        <v>10</v>
+      </c>
       <c r="I28" s="47" t="n"/>
       <c r="J28" s="48" t="n"/>
-      <c r="K28" s="49" t="n"/>
-      <c r="L28" s="46" t="n"/>
-      <c r="M28" s="46" t="n"/>
-      <c r="N28" s="46" t="n"/>
+      <c r="K28" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="L28" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M28" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N28" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O28" s="50" t="n"/>
       <c r="P28" s="51" t="n"/>
       <c r="Q28" s="39">
@@ -18369,7 +19063,11 @@
         <v/>
       </c>
       <c r="T28" s="91" t="n"/>
-      <c r="U28" s="52" t="n"/>
+      <c r="U28" s="52" t="inlineStr">
+        <is>
+          <t>Marvel</t>
+        </is>
+      </c>
       <c r="V28" s="0">
         <f>IF(B28="","",IFERROR(VLOOKUP(C28,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B28,B28),"000"),""))</f>
         <v/>
@@ -18380,19 +19078,57 @@
         <f>IF(T29="","",IMAGE(T29,4,50,50))</f>
         <v/>
       </c>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="E29" s="34" t="n"/>
-      <c r="F29" s="35" t="n"/>
-      <c r="G29" s="34" t="n"/>
-      <c r="H29" s="35" t="n"/>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Baby Groot</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Verde e Marrom</t>
+        </is>
+      </c>
+      <c r="E29" s="34" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="F29" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G29" s="34" t="inlineStr">
+        <is>
+          <t>Marrom</t>
+        </is>
+      </c>
+      <c r="H29" s="35" t="n">
+        <v>5</v>
+      </c>
       <c r="I29" s="34" t="n"/>
       <c r="J29" s="35" t="n"/>
-      <c r="K29" s="36" t="n"/>
-      <c r="L29" s="33" t="n"/>
-      <c r="M29" s="33" t="n"/>
-      <c r="N29" s="33" t="n"/>
+      <c r="K29" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="L29" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M29" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N29" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O29" s="37" t="n"/>
       <c r="P29" s="38" t="n"/>
       <c r="Q29" s="39">
@@ -18408,7 +19144,11 @@
         <v/>
       </c>
       <c r="T29" s="91" t="n"/>
-      <c r="U29" s="43" t="n"/>
+      <c r="U29" s="43" t="inlineStr">
+        <is>
+          <t>Marvel</t>
+        </is>
+      </c>
       <c r="V29" s="0">
         <f>IF(B29="","",IFERROR(VLOOKUP(C29,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B29,B29),"000"),""))</f>
         <v/>
@@ -18419,19 +19159,51 @@
         <f>IF(T30="","",IMAGE(T30,4,50,50))</f>
         <v/>
       </c>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="47" t="n"/>
-      <c r="F30" s="48" t="n"/>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Alien</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="E30" s="47" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="F30" s="48" t="n">
+        <v>16</v>
+      </c>
       <c r="G30" s="47" t="n"/>
       <c r="H30" s="48" t="n"/>
       <c r="I30" s="47" t="n"/>
       <c r="J30" s="48" t="n"/>
-      <c r="K30" s="49" t="n"/>
-      <c r="L30" s="46" t="n"/>
-      <c r="M30" s="46" t="n"/>
-      <c r="N30" s="46" t="n"/>
+      <c r="K30" s="49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L30" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M30" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N30" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O30" s="50" t="n"/>
       <c r="P30" s="51" t="n"/>
       <c r="Q30" s="39">
@@ -18458,19 +19230,63 @@
         <f>IF(T31="","",IMAGE(T31,4,50,50))</f>
         <v/>
       </c>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
-      <c r="E31" s="34" t="n"/>
-      <c r="F31" s="35" t="n"/>
-      <c r="G31" s="34" t="n"/>
-      <c r="H31" s="35" t="n"/>
-      <c r="I31" s="34" t="n"/>
-      <c r="J31" s="35" t="n"/>
-      <c r="K31" s="36" t="n"/>
-      <c r="L31" s="33" t="n"/>
-      <c r="M31" s="33" t="n"/>
-      <c r="N31" s="33" t="n"/>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Harry Potter</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="E31" s="34" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="F31" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="G31" s="34" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="H31" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="I31" s="34" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="J31" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="K31" s="36" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L31" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M31" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N31" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O31" s="37" t="n"/>
       <c r="P31" s="38" t="n"/>
       <c r="Q31" s="39">
@@ -18497,19 +19313,57 @@
         <f>IF(T32="","",IMAGE(T32,4,50,50))</f>
         <v/>
       </c>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="47" t="n"/>
-      <c r="F32" s="48" t="n"/>
-      <c r="G32" s="47" t="n"/>
-      <c r="H32" s="48" t="n"/>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Cone</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Laranja e Amarelo</t>
+        </is>
+      </c>
+      <c r="E32" s="47" t="inlineStr">
+        <is>
+          <t>Laranja</t>
+        </is>
+      </c>
+      <c r="F32" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="G32" s="47" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="H32" s="48" t="n">
+        <v>8</v>
+      </c>
       <c r="I32" s="47" t="n"/>
       <c r="J32" s="48" t="n"/>
-      <c r="K32" s="49" t="n"/>
-      <c r="L32" s="46" t="n"/>
-      <c r="M32" s="46" t="n"/>
-      <c r="N32" s="46" t="n"/>
+      <c r="K32" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M32" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N32" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O32" s="50" t="n"/>
       <c r="P32" s="51" t="n"/>
       <c r="Q32" s="39">
@@ -18525,7 +19379,11 @@
         <v/>
       </c>
       <c r="T32" s="91" t="n"/>
-      <c r="U32" s="52" t="n"/>
+      <c r="U32" s="52" t="inlineStr">
+        <is>
+          <t>Peça sensorial cone</t>
+        </is>
+      </c>
       <c r="V32" s="0">
         <f>IF(B32="","",IFERROR(VLOOKUP(C32,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B32,B32),"000"),""))</f>
         <v/>
@@ -18536,19 +19394,57 @@
         <f>IF(T33="","",IMAGE(T33,4,50,50))</f>
         <v/>
       </c>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
-      <c r="E33" s="34" t="n"/>
-      <c r="F33" s="35" t="n"/>
-      <c r="G33" s="34" t="n"/>
-      <c r="H33" s="35" t="n"/>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Pokebola</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Vermelho e Branco</t>
+        </is>
+      </c>
+      <c r="E33" s="34" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="F33" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="G33" s="34" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="H33" s="35" t="n">
+        <v>4</v>
+      </c>
       <c r="I33" s="34" t="n"/>
       <c r="J33" s="35" t="n"/>
-      <c r="K33" s="36" t="n"/>
-      <c r="L33" s="33" t="n"/>
-      <c r="M33" s="33" t="n"/>
-      <c r="N33" s="33" t="n"/>
+      <c r="K33" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M33" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N33" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O33" s="37" t="n"/>
       <c r="P33" s="38" t="n"/>
       <c r="Q33" s="39">
@@ -18564,7 +19460,11 @@
         <v/>
       </c>
       <c r="T33" s="91" t="n"/>
-      <c r="U33" s="43" t="n"/>
+      <c r="U33" s="43" t="inlineStr">
+        <is>
+          <t>Pokémon</t>
+        </is>
+      </c>
       <c r="V33" s="0">
         <f>IF(B33="","",IFERROR(VLOOKUP(C33,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B33,B33),"000"),""))</f>
         <v/>
@@ -18575,19 +19475,51 @@
         <f>IF(T34="","",IMAGE(T34,4,50,50))</f>
         <v/>
       </c>
-      <c r="B34" s="12" t="n"/>
-      <c r="C34" s="12" t="n"/>
-      <c r="D34" s="12" t="n"/>
-      <c r="E34" s="47" t="n"/>
-      <c r="F34" s="48" t="n"/>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>Fantasma Vermelho</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="E34" s="47" t="inlineStr">
+        <is>
+          <t>Vermelho</t>
+        </is>
+      </c>
+      <c r="F34" s="48" t="n">
+        <v>10</v>
+      </c>
       <c r="G34" s="47" t="n"/>
       <c r="H34" s="48" t="n"/>
       <c r="I34" s="47" t="n"/>
       <c r="J34" s="48" t="n"/>
-      <c r="K34" s="49" t="n"/>
-      <c r="L34" s="46" t="n"/>
-      <c r="M34" s="46" t="n"/>
-      <c r="N34" s="46" t="n"/>
+      <c r="K34" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M34" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N34" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O34" s="50" t="n"/>
       <c r="P34" s="51" t="n"/>
       <c r="Q34" s="39">
@@ -18603,7 +19535,11 @@
         <v/>
       </c>
       <c r="T34" s="91" t="n"/>
-      <c r="U34" s="52" t="n"/>
+      <c r="U34" s="52" t="inlineStr">
+        <is>
+          <t>Pac-Man</t>
+        </is>
+      </c>
       <c r="V34" s="0">
         <f>IF(B34="","",IFERROR(VLOOKUP(C34,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B34,B34),"000"),""))</f>
         <v/>
@@ -18614,19 +19550,57 @@
         <f>IF(T35="","",IMAGE(T35,4,50,50))</f>
         <v/>
       </c>
-      <c r="B35" s="8" t="n"/>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="8" t="n"/>
-      <c r="E35" s="34" t="n"/>
-      <c r="F35" s="35" t="n"/>
-      <c r="G35" s="34" t="n"/>
-      <c r="H35" s="35" t="n"/>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Dado RPG</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="E35" s="34" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="F35" s="35" t="n">
+        <v>8</v>
+      </c>
+      <c r="G35" s="34" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="H35" s="35" t="n">
+        <v>2</v>
+      </c>
       <c r="I35" s="34" t="n"/>
       <c r="J35" s="35" t="n"/>
-      <c r="K35" s="36" t="n"/>
-      <c r="L35" s="33" t="n"/>
-      <c r="M35" s="33" t="n"/>
-      <c r="N35" s="33" t="n"/>
+      <c r="K35" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M35" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N35" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O35" s="37" t="n"/>
       <c r="P35" s="38" t="n"/>
       <c r="Q35" s="39">
@@ -18642,7 +19616,11 @@
         <v/>
       </c>
       <c r="T35" s="91" t="n"/>
-      <c r="U35" s="43" t="n"/>
+      <c r="U35" s="43" t="inlineStr">
+        <is>
+          <t>Dado 3D RPG</t>
+        </is>
+      </c>
       <c r="V35" s="0">
         <f>IF(B35="","",IFERROR(VLOOKUP(C35,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B35,B35),"000"),""))</f>
         <v/>
@@ -18653,19 +19631,51 @@
         <f>IF(T36="","",IMAGE(T36,4,50,50))</f>
         <v/>
       </c>
-      <c r="B36" s="12" t="n"/>
-      <c r="C36" s="12" t="n"/>
-      <c r="D36" s="12" t="n"/>
-      <c r="E36" s="47" t="n"/>
-      <c r="F36" s="48" t="n"/>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>Mala</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>Marrom</t>
+        </is>
+      </c>
+      <c r="E36" s="47" t="inlineStr">
+        <is>
+          <t>Marrom</t>
+        </is>
+      </c>
+      <c r="F36" s="48" t="n">
+        <v>14</v>
+      </c>
       <c r="G36" s="47" t="n"/>
       <c r="H36" s="48" t="n"/>
       <c r="I36" s="47" t="n"/>
       <c r="J36" s="48" t="n"/>
-      <c r="K36" s="49" t="n"/>
-      <c r="L36" s="46" t="n"/>
-      <c r="M36" s="46" t="n"/>
-      <c r="N36" s="46" t="n"/>
+      <c r="K36" s="49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L36" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M36" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N36" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O36" s="50" t="n"/>
       <c r="P36" s="51" t="n"/>
       <c r="Q36" s="39">
@@ -18692,19 +19702,51 @@
         <f>IF(T37="","",IMAGE(T37,4,50,50))</f>
         <v/>
       </c>
-      <c r="B37" s="8" t="n"/>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="8" t="n"/>
-      <c r="E37" s="34" t="n"/>
-      <c r="F37" s="35" t="n"/>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Jacaré</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="E37" s="34" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="F37" s="35" t="n">
+        <v>18</v>
+      </c>
       <c r="G37" s="34" t="n"/>
       <c r="H37" s="35" t="n"/>
       <c r="I37" s="34" t="n"/>
       <c r="J37" s="35" t="n"/>
-      <c r="K37" s="36" t="n"/>
-      <c r="L37" s="33" t="n"/>
-      <c r="M37" s="33" t="n"/>
-      <c r="N37" s="33" t="n"/>
+      <c r="K37" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="L37" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M37" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N37" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O37" s="37" t="n"/>
       <c r="P37" s="38" t="n"/>
       <c r="Q37" s="39">
@@ -18731,19 +19773,51 @@
         <f>IF(T38="","",IMAGE(T38,4,50,50))</f>
         <v/>
       </c>
-      <c r="B38" s="12" t="n"/>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="12" t="n"/>
-      <c r="E38" s="47" t="n"/>
-      <c r="F38" s="48" t="n"/>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Bloco de Interrogação Mario</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="E38" s="47" t="inlineStr">
+        <is>
+          <t>Amarelo</t>
+        </is>
+      </c>
+      <c r="F38" s="48" t="n">
+        <v>15</v>
+      </c>
       <c r="G38" s="47" t="n"/>
       <c r="H38" s="48" t="n"/>
       <c r="I38" s="47" t="n"/>
       <c r="J38" s="48" t="n"/>
-      <c r="K38" s="49" t="n"/>
-      <c r="L38" s="46" t="n"/>
-      <c r="M38" s="46" t="n"/>
-      <c r="N38" s="46" t="n"/>
+      <c r="K38" s="49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L38" s="46" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M38" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N38" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O38" s="50" t="n"/>
       <c r="P38" s="51" t="n"/>
       <c r="Q38" s="39">
@@ -18759,7 +19833,11 @@
         <v/>
       </c>
       <c r="T38" s="91" t="n"/>
-      <c r="U38" s="52" t="n"/>
+      <c r="U38" s="52" t="inlineStr">
+        <is>
+          <t>Super Mario</t>
+        </is>
+      </c>
       <c r="V38" s="0">
         <f>IF(B38="","",IFERROR(VLOOKUP(C38,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B38,B38),"000"),""))</f>
         <v/>
@@ -18770,19 +19848,57 @@
         <f>IF(T39="","",IMAGE(T39,4,50,50))</f>
         <v/>
       </c>
-      <c r="B39" s="8" t="n"/>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="8" t="n"/>
-      <c r="E39" s="34" t="n"/>
-      <c r="F39" s="35" t="n"/>
-      <c r="G39" s="34" t="n"/>
-      <c r="H39" s="35" t="n"/>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Boca Abridor de Garrafa</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Plaquinha</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Variado</t>
+        </is>
+      </c>
+      <c r="E39" s="34" t="inlineStr">
+        <is>
+          <t>Preto</t>
+        </is>
+      </c>
+      <c r="F39" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G39" s="34" t="inlineStr">
+        <is>
+          <t>Branco</t>
+        </is>
+      </c>
+      <c r="H39" s="35" t="n">
+        <v>5</v>
+      </c>
       <c r="I39" s="34" t="n"/>
       <c r="J39" s="35" t="n"/>
-      <c r="K39" s="36" t="n"/>
-      <c r="L39" s="33" t="n"/>
-      <c r="M39" s="33" t="n"/>
-      <c r="N39" s="33" t="n"/>
+      <c r="K39" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="L39" s="33" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="M39" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="N39" s="33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
       <c r="O39" s="37" t="n"/>
       <c r="P39" s="38" t="n"/>
       <c r="Q39" s="39">
@@ -18798,7 +19914,11 @@
         <v/>
       </c>
       <c r="T39" s="91" t="n"/>
-      <c r="U39" s="43" t="n"/>
+      <c r="U39" s="43" t="inlineStr">
+        <is>
+          <t>Abridor de garrafa — boca</t>
+        </is>
+      </c>
       <c r="V39" s="0">
         <f>IF(B39="","",IFERROR(VLOOKUP(C39,'⚙️ Parâmetros'!$A$20:$B$29,2,0)&amp;"-2026-"&amp;TEXT(COUNTIF($B$7:B39,B39),"000"),""))</f>
         <v/>
@@ -45232,12 +46352,29 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" s="109">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="33" t="n"/>
-      <c r="E5" s="33" t="n"/>
-      <c r="F5" s="33" t="n"/>
+      <c r="A5" s="8">
+        <f>IF(B5="","",IFERROR(VLOOKUP(B5,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Estádio Corinthians</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="n">
+        <v>29</v>
+      </c>
+      <c r="E5" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G5" s="77">
         <f>IF(A5="","",D5-E5-F5)</f>
         <v/>
@@ -45248,12 +46385,29 @@
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" s="109">
-      <c r="A6" s="12" t="n"/>
-      <c r="B6" s="12" t="n"/>
-      <c r="C6" s="12" t="n"/>
-      <c r="D6" s="46" t="n"/>
-      <c r="E6" s="46" t="n"/>
-      <c r="F6" s="46" t="n"/>
+      <c r="A6" s="12">
+        <f>IF(B6="","",IFERROR(VLOOKUP(B6,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Estádio Palmeiras</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D6" s="46" t="n">
+        <v>14</v>
+      </c>
+      <c r="E6" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G6" s="77">
         <f>IF(A6="","",D6-E6-F6)</f>
         <v/>
@@ -45264,12 +46418,29 @@
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="109">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="33" t="n"/>
-      <c r="E7" s="33" t="n"/>
-      <c r="F7" s="33" t="n"/>
+      <c r="A7" s="8">
+        <f>IF(B7="","",IFERROR(VLOOKUP(B7,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Estádio São Paulo</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G7" s="77">
         <f>IF(A7="","",D7-E7-F7)</f>
         <v/>
@@ -45280,12 +46451,29 @@
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="109">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="46" t="n"/>
-      <c r="E8" s="46" t="n"/>
-      <c r="F8" s="46" t="n"/>
+      <c r="A8" s="12">
+        <f>IF(B8="","",IFERROR(VLOOKUP(B8,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Martelo Thor</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D8" s="46" t="n">
+        <v>31</v>
+      </c>
+      <c r="E8" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G8" s="77">
         <f>IF(A8="","",D8-E8-F8)</f>
         <v/>
@@ -45296,12 +46484,29 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" s="109">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="33" t="n"/>
-      <c r="E9" s="33" t="n"/>
-      <c r="F9" s="33" t="n"/>
+      <c r="A9" s="8">
+        <f>IF(B9="","",IFERROR(VLOOKUP(B9,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Estádio Santos</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G9" s="77">
         <f>IF(A9="","",D9-E9-F9)</f>
         <v/>
@@ -45312,12 +46517,29 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" s="109">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="46" t="n"/>
-      <c r="E10" s="46" t="n"/>
-      <c r="F10" s="46" t="n"/>
+      <c r="A10" s="12">
+        <f>IF(B10="","",IFERROR(VLOOKUP(B10,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Estádio Flamengo</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D10" s="46" t="n">
+        <v>14</v>
+      </c>
+      <c r="E10" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G10" s="77">
         <f>IF(A10="","",D10-E10-F10)</f>
         <v/>
@@ -45328,12 +46550,29 @@
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="109">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="33" t="n"/>
-      <c r="E11" s="33" t="n"/>
-      <c r="F11" s="33" t="n"/>
+      <c r="A11" s="8">
+        <f>IF(B11="","",IFERROR(VLOOKUP(B11,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Escudo Flamengo</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" s="77">
         <f>IF(A11="","",D11-E11-F11)</f>
         <v/>
@@ -45344,12 +46583,29 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="109">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="46" t="n"/>
-      <c r="E12" s="46" t="n"/>
-      <c r="F12" s="46" t="n"/>
+      <c r="A12" s="12">
+        <f>IF(B12="","",IFERROR(VLOOKUP(B12,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Estela Sensorial Maior</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D12" s="46" t="n">
+        <v>9</v>
+      </c>
+      <c r="E12" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G12" s="77">
         <f>IF(A12="","",D12-E12-F12)</f>
         <v/>
@@ -45360,12 +46616,29 @@
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" s="109">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="33" t="n"/>
-      <c r="E13" s="33" t="n"/>
-      <c r="F13" s="33" t="n"/>
+      <c r="A13" s="8">
+        <f>IF(B13="","",IFERROR(VLOOKUP(B13,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Minicraft Verde</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="n">
+        <v>26</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G13" s="77">
         <f>IF(A13="","",D13-E13-F13)</f>
         <v/>
@@ -45376,12 +46649,29 @@
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" s="109">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="46" t="n"/>
-      <c r="E14" s="46" t="n"/>
-      <c r="F14" s="46" t="n"/>
+      <c r="A14" s="12">
+        <f>IF(B14="","",IFERROR(VLOOKUP(B14,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Pentágono Sensorial</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="n">
+        <v>23</v>
+      </c>
+      <c r="E14" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G14" s="77">
         <f>IF(A14="","",D14-E14-F14)</f>
         <v/>
@@ -45392,12 +46682,29 @@
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" s="109">
-      <c r="A15" s="8" t="n"/>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="33" t="n"/>
-      <c r="E15" s="33" t="n"/>
-      <c r="F15" s="33" t="n"/>
+      <c r="A15" s="8">
+        <f>IF(B15="","",IFERROR(VLOOKUP(B15,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Tubarão</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="n">
+        <v>29</v>
+      </c>
+      <c r="E15" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" s="77">
         <f>IF(A15="","",D15-E15-F15)</f>
         <v/>
@@ -45408,12 +46715,29 @@
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" s="109">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="46" t="n"/>
-      <c r="E16" s="46" t="n"/>
-      <c r="F16" s="46" t="n"/>
+      <c r="A16" s="12">
+        <f>IF(B16="","",IFERROR(VLOOKUP(B16,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Nossa Senhora</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D16" s="46" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G16" s="77">
         <f>IF(A16="","",D16-E16-F16)</f>
         <v/>
@@ -45424,12 +46748,29 @@
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" s="109">
-      <c r="A17" s="8" t="n"/>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="33" t="n"/>
-      <c r="E17" s="33" t="n"/>
-      <c r="F17" s="33" t="n"/>
+      <c r="A17" s="8">
+        <f>IF(B17="","",IFERROR(VLOOKUP(B17,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Gato Preto</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="n">
+        <v>20</v>
+      </c>
+      <c r="E17" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G17" s="77">
         <f>IF(A17="","",D17-E17-F17)</f>
         <v/>
@@ -45440,12 +46781,29 @@
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="109">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="46" t="n"/>
-      <c r="E18" s="46" t="n"/>
-      <c r="F18" s="46" t="n"/>
+      <c r="A18" s="12">
+        <f>IF(B18="","",IFERROR(VLOOKUP(B18,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Stormtrooper</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D18" s="46" t="n">
+        <v>11</v>
+      </c>
+      <c r="E18" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G18" s="77">
         <f>IF(A18="","",D18-E18-F18)</f>
         <v/>
@@ -45456,12 +46814,29 @@
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="109">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="33" t="n"/>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="33" t="n"/>
+      <c r="A19" s="8">
+        <f>IF(B19="","",IFERROR(VLOOKUP(B19,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Polvo</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D19" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="E19" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G19" s="77">
         <f>IF(A19="","",D19-E19-F19)</f>
         <v/>
@@ -45472,12 +46847,29 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" s="109">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="46" t="n"/>
-      <c r="E20" s="46" t="n"/>
-      <c r="F20" s="46" t="n"/>
+      <c r="A20" s="12">
+        <f>IF(B20="","",IFERROR(VLOOKUP(B20,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Copo Stanley</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D20" s="46" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G20" s="77">
         <f>IF(A20="","",D20-E20-F20)</f>
         <v/>
@@ -45488,12 +46880,29 @@
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" s="109">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="33" t="n"/>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="33" t="n"/>
+      <c r="A21" s="8">
+        <f>IF(B21="","",IFERROR(VLOOKUP(B21,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Homem de Ferro</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="E21" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G21" s="77">
         <f>IF(A21="","",D21-E21-F21)</f>
         <v/>
@@ -45504,12 +46913,29 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" s="109">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="46" t="n"/>
-      <c r="E22" s="46" t="n"/>
-      <c r="F22" s="46" t="n"/>
+      <c r="A22" s="12">
+        <f>IF(B22="","",IFERROR(VLOOKUP(B22,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Homem Aranha</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D22" s="46" t="n">
+        <v>18</v>
+      </c>
+      <c r="E22" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G22" s="77">
         <f>IF(A22="","",D22-E22-F22)</f>
         <v/>
@@ -45520,12 +46946,29 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="109">
-      <c r="A23" s="8" t="n"/>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="33" t="n"/>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="33" t="n"/>
+      <c r="A23" s="8">
+        <f>IF(B23="","",IFERROR(VLOOKUP(B23,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Baby Groot</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G23" s="77">
         <f>IF(A23="","",D23-E23-F23)</f>
         <v/>
@@ -45536,12 +46979,29 @@
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="109">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="46" t="n"/>
-      <c r="E24" s="46" t="n"/>
-      <c r="F24" s="46" t="n"/>
+      <c r="A24" s="12">
+        <f>IF(B24="","",IFERROR(VLOOKUP(B24,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Alien</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D24" s="46" t="n">
+        <v>20</v>
+      </c>
+      <c r="E24" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G24" s="77">
         <f>IF(A24="","",D24-E24-F24)</f>
         <v/>
@@ -45552,12 +47012,29 @@
       </c>
     </row>
     <row r="25" ht="18" customHeight="1" s="109">
-      <c r="A25" s="8" t="n"/>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="33" t="n"/>
-      <c r="E25" s="33" t="n"/>
-      <c r="F25" s="33" t="n"/>
+      <c r="A25" s="8">
+        <f>IF(B25="","",IFERROR(VLOOKUP(B25,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Harry Potter</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="n">
+        <v>11</v>
+      </c>
+      <c r="E25" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G25" s="77">
         <f>IF(A25="","",D25-E25-F25)</f>
         <v/>
@@ -45568,12 +47045,29 @@
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="109">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="46" t="n"/>
-      <c r="E26" s="46" t="n"/>
-      <c r="F26" s="46" t="n"/>
+      <c r="A26" s="12">
+        <f>IF(B26="","",IFERROR(VLOOKUP(B26,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Cone</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D26" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G26" s="77">
         <f>IF(A26="","",D26-E26-F26)</f>
         <v/>
@@ -45584,12 +47078,29 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="109">
-      <c r="A27" s="8" t="n"/>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="33" t="n"/>
-      <c r="E27" s="33" t="n"/>
-      <c r="F27" s="33" t="n"/>
+      <c r="A27" s="8">
+        <f>IF(B27="","",IFERROR(VLOOKUP(B27,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Pokebola</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D27" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G27" s="77">
         <f>IF(A27="","",D27-E27-F27)</f>
         <v/>
@@ -45600,12 +47111,29 @@
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="109">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="46" t="n"/>
-      <c r="E28" s="46" t="n"/>
-      <c r="F28" s="46" t="n"/>
+      <c r="A28" s="12">
+        <f>IF(B28="","",IFERROR(VLOOKUP(B28,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Fantasma Vermelho</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D28" s="46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E28" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G28" s="77">
         <f>IF(A28="","",D28-E28-F28)</f>
         <v/>
@@ -45616,12 +47144,29 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" s="109">
-      <c r="A29" s="8" t="n"/>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="33" t="n"/>
-      <c r="E29" s="33" t="n"/>
-      <c r="F29" s="33" t="n"/>
+      <c r="A29" s="8">
+        <f>IF(B29="","",IFERROR(VLOOKUP(B29,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Dado RPG</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Enfeite/Decoração</t>
+        </is>
+      </c>
+      <c r="D29" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G29" s="77">
         <f>IF(A29="","",D29-E29-F29)</f>
         <v/>
@@ -45632,12 +47177,29 @@
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="109">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="46" t="n"/>
-      <c r="E30" s="46" t="n"/>
-      <c r="F30" s="46" t="n"/>
+      <c r="A30" s="12">
+        <f>IF(B30="","",IFERROR(VLOOKUP(B30,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Mala</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D30" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G30" s="77">
         <f>IF(A30="","",D30-E30-F30)</f>
         <v/>
@@ -45648,12 +47210,29 @@
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="109">
-      <c r="A31" s="8" t="n"/>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="33" t="n"/>
-      <c r="E31" s="33" t="n"/>
-      <c r="F31" s="33" t="n"/>
+      <c r="A31" s="8">
+        <f>IF(B31="","",IFERROR(VLOOKUP(B31,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Jacaré</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D31" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G31" s="77">
         <f>IF(A31="","",D31-E31-F31)</f>
         <v/>
@@ -45664,12 +47243,29 @@
       </c>
     </row>
     <row r="32" ht="18" customHeight="1" s="109">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="46" t="n"/>
-      <c r="E32" s="46" t="n"/>
-      <c r="F32" s="46" t="n"/>
+      <c r="A32" s="12">
+        <f>IF(B32="","",IFERROR(VLOOKUP(B32,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Bloco de Interrogação Mario</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Miniatura</t>
+        </is>
+      </c>
+      <c r="D32" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="46" t="n">
+        <v>0</v>
+      </c>
       <c r="G32" s="77">
         <f>IF(A32="","",D32-E32-F32)</f>
         <v/>
@@ -45680,12 +47276,29 @@
       </c>
     </row>
     <row r="33" ht="18" customHeight="1" s="109">
-      <c r="A33" s="8" t="n"/>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="33" t="n"/>
-      <c r="E33" s="33" t="n"/>
-      <c r="F33" s="33" t="n"/>
+      <c r="A33" s="8">
+        <f>IF(B33="","",IFERROR(VLOOKUP(B33,'📋 Catálogo'!$B$7:$V$41,21,0),""))</f>
+        <v/>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Boca Abridor de Garrafa</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Plaquinha</t>
+        </is>
+      </c>
+      <c r="D33" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="E33" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="33" t="n">
+        <v>0</v>
+      </c>
       <c r="G33" s="77">
         <f>IF(A33="","",D33-E33-F33)</f>
         <v/>

</xml_diff>